<commit_message>
docs(catatan-dev-team): pisahkan kolom H (path API) & kolom I (keterangan) di sheet Web
</commit_message>
<xml_diff>
--- a/docs/api-mapping/catatan-dev-team.xlsx
+++ b/docs/api-mapping/catatan-dev-team.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1021"/>
+  <dimension ref="A1:I1021"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="2.63" customWidth="1" style="17" min="1" max="1"/>
@@ -432,7 +432,8 @@
     <col width="23.88" customWidth="1" style="17" min="5" max="5"/>
     <col width="15.75" customWidth="1" style="17" min="6" max="6"/>
     <col width="13" customWidth="1" style="17" min="7" max="7"/>
-    <col width="58" customWidth="1" style="17" min="8" max="8"/>
+    <col width="52" customWidth="1" style="17" min="8" max="8"/>
+    <col width="52" customWidth="1" style="17" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -457,7 +458,12 @@
       </c>
       <c r="H1" s="18" t="inlineStr">
         <is>
-          <t>Endpoint BMKG (hasil scrapping baseline)</t>
+          <t>Endpoint BMKG (path)</t>
+        </is>
+      </c>
+      <c r="I1" s="18" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
         </is>
       </c>
     </row>
@@ -528,7 +534,12 @@
       </c>
       <c r="H4" s="20" t="inlineStr">
         <is>
-          <t>GET /api/df/v1/adm/coord (GPS→alamat admin) — sudah dipakai redesign</t>
+          <t>GET /api/df/v1/adm/coord</t>
+        </is>
+      </c>
+      <c r="I4" s="20" t="inlineStr">
+        <is>
+          <t>GPS → alamat admin; sudah dipakai redesign</t>
         </is>
       </c>
     </row>
@@ -561,7 +572,12 @@
       </c>
       <c r="H5" s="20" t="inlineStr">
         <is>
-          <t>lokasi.timezone dari /api/df/v1/forecast/coord</t>
+          <t>GET /api/df/v1/forecast/coord</t>
+        </is>
+      </c>
+      <c r="I5" s="20" t="inlineStr">
+        <is>
+          <t>field lokasi.timezone (deteksi WIB/WITA/WIT)</t>
         </is>
       </c>
     </row>
@@ -590,7 +606,12 @@
       </c>
       <c r="H6" s="20" t="inlineStr">
         <is>
-          <t>GET /api/presentwx/coord (observasi) + /api/df/v1/forecast/coord</t>
+          <t>GET /api/presentwx/coord</t>
+        </is>
+      </c>
+      <c r="I6" s="20" t="inlineStr">
+        <is>
+          <t>observasi aktual kartu kondisi saat ini</t>
         </is>
       </c>
     </row>
@@ -616,6 +637,11 @@
       </c>
       <c r="H7" s="20" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I7" s="20" t="inlineStr">
+        <is>
           <t>Tidak terdeteksi di baseline (form laporan, tanpa XHR)</t>
         </is>
       </c>
@@ -649,6 +675,11 @@
       </c>
       <c r="H8" s="20" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I8" s="20" t="inlineStr">
+        <is>
           <t>Statis (link App Store/Play Store)</t>
         </is>
       </c>
@@ -682,7 +713,12 @@
       </c>
       <c r="H9" s="20" t="inlineStr">
         <is>
-          <t>GET /api/df/v1/forecast/coord + /api/presentwx/coord per koordinat kota</t>
+          <t>GET /api/df/v1/forecast/coord + GET /api/presentwx/coord</t>
+        </is>
+      </c>
+      <c r="I9" s="20" t="inlineStr">
+        <is>
+          <t>per koordinat kota</t>
         </is>
       </c>
     </row>
@@ -715,6 +751,11 @@
       </c>
       <c r="H10" s="20" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I10" s="20" t="inlineStr">
+        <is>
           <t>Tidak ada endpoint khusus — dihitung klien dari presentwx (t, hu, ws)</t>
         </is>
       </c>
@@ -748,7 +789,12 @@
       </c>
       <c r="H11" s="20" t="inlineStr">
         <is>
-          <t>Tidak ada JSON AQI — hanya tile polusi /api/v1/spartan/pollution/{pol}/...</t>
+          <t>GET /api/v1/spartan/pollution/{pol}/{lvl}/{t0}/{t1}/{z}/{x}/{y}.png</t>
+        </is>
+      </c>
+      <c r="I11" s="20" t="inlineStr">
+        <is>
+          <t>Tidak ada JSON AQI — hanya tile polusi untuk peta</t>
         </is>
       </c>
     </row>
@@ -777,7 +823,12 @@
       </c>
       <c r="H12" s="20" t="inlineStr">
         <is>
-          <t>GET /api/presentwx/coord: t (suhu), ws (angin), wd (arah), hu (kelembapan)</t>
+          <t>GET /api/presentwx/coord</t>
+        </is>
+      </c>
+      <c r="I12" s="20" t="inlineStr">
+        <is>
+          <t>sumber parameter: t, ws, wd, hu</t>
         </is>
       </c>
     </row>
@@ -803,7 +854,12 @@
       </c>
       <c r="H13" s="20" t="inlineStr">
         <is>
-          <t>GET /api/presentwx/coord → t</t>
+          <t>GET /api/presentwx/coord</t>
+        </is>
+      </c>
+      <c r="I13" s="20" t="inlineStr">
+        <is>
+          <t>field t (°C)</t>
         </is>
       </c>
     </row>
@@ -829,7 +885,12 @@
       </c>
       <c r="H14" s="20" t="inlineStr">
         <is>
-          <t>GET /api/presentwx/coord → ws</t>
+          <t>GET /api/presentwx/coord</t>
+        </is>
+      </c>
+      <c r="I14" s="20" t="inlineStr">
+        <is>
+          <t>field ws (km/h)</t>
         </is>
       </c>
     </row>
@@ -855,7 +916,12 @@
       </c>
       <c r="H15" s="20" t="inlineStr">
         <is>
-          <t>GET /api/presentwx/coord → wd / wd_deg</t>
+          <t>GET /api/presentwx/coord</t>
+        </is>
+      </c>
+      <c r="I15" s="20" t="inlineStr">
+        <is>
+          <t>field wd / wd_deg</t>
         </is>
       </c>
     </row>
@@ -881,7 +947,12 @@
       </c>
       <c r="H16" s="20" t="inlineStr">
         <is>
-          <t>GET /api/presentwx/coord → hu</t>
+          <t>GET /api/presentwx/coord</t>
+        </is>
+      </c>
+      <c r="I16" s="20" t="inlineStr">
+        <is>
+          <t>field hu (%)</t>
         </is>
       </c>
     </row>
@@ -914,6 +985,11 @@
       </c>
       <c r="H17" s="20" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I17" s="20" t="inlineStr">
+        <is>
           <t>Tidak ada (fitur investigasi, tanpa API)</t>
         </is>
       </c>
@@ -943,7 +1019,12 @@
       </c>
       <c r="H18" s="20" t="inlineStr">
         <is>
-          <t>GET /api/df/v1/forecast/coord → data[0].cuaca[0] (hourly)</t>
+          <t>GET /api/df/v1/forecast/coord</t>
+        </is>
+      </c>
+      <c r="I18" s="20" t="inlineStr">
+        <is>
+          <t>data[0].cuaca[0] = grup hourly</t>
         </is>
       </c>
     </row>
@@ -969,7 +1050,12 @@
       </c>
       <c r="H19" s="20" t="inlineStr">
         <is>
-          <t>forecast/coord → t per jam</t>
+          <t>GET /api/df/v1/forecast/coord</t>
+        </is>
+      </c>
+      <c r="I19" s="20" t="inlineStr">
+        <is>
+          <t>field t per jam</t>
         </is>
       </c>
     </row>
@@ -995,7 +1081,12 @@
       </c>
       <c r="H20" s="20" t="inlineStr">
         <is>
-          <t>forecast/coord → tp (mm) per jam</t>
+          <t>GET /api/df/v1/forecast/coord</t>
+        </is>
+      </c>
+      <c r="I20" s="20" t="inlineStr">
+        <is>
+          <t>field tp (mm) per jam</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1112,12 @@
       </c>
       <c r="H21" s="20" t="inlineStr">
         <is>
-          <t>forecast/coord → ws per jam</t>
+          <t>GET /api/df/v1/forecast/coord</t>
+        </is>
+      </c>
+      <c r="I21" s="20" t="inlineStr">
+        <is>
+          <t>field ws per jam</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1143,12 @@
       </c>
       <c r="H22" s="20" t="inlineStr">
         <is>
-          <t>forecast/coord → hu per jam</t>
+          <t>GET /api/df/v1/forecast/coord</t>
+        </is>
+      </c>
+      <c r="I22" s="20" t="inlineStr">
+        <is>
+          <t>field hu per jam</t>
         </is>
       </c>
     </row>
@@ -1073,6 +1174,11 @@
       </c>
       <c r="H23" s="20" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I23" s="20" t="inlineStr">
+        <is>
           <t>Tidak ada JSON AQ per jam (hanya tile polusi)</t>
         </is>
       </c>
@@ -1101,6 +1207,11 @@
         </is>
       </c>
       <c r="H24" s="20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I24" s="20" t="inlineStr">
         <is>
           <t>Lihat per sub-aktivitas</t>
         </is>
@@ -1128,6 +1239,11 @@
       </c>
       <c r="H25" s="20" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I25" s="20" t="inlineStr">
+        <is>
           <t>Tidak terdeteksi di baseline (redesign pakai Overpass OSM)</t>
         </is>
       </c>
@@ -1154,7 +1270,12 @@
       </c>
       <c r="H26" s="20" t="inlineStr">
         <is>
-          <t>/api/v1/public/maritim/nearest-location (wilayah laut terdekat)</t>
+          <t>GET /api/v1/public/maritim/nearest-location</t>
+        </is>
+      </c>
+      <c r="I26" s="20" t="inlineStr">
+        <is>
+          <t>wilayah laut terdekat (code, name, wilpel, polygon)</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1301,12 @@
       </c>
       <c r="H27" s="20" t="inlineStr">
         <is>
-          <t>/api/v1/maritim/route + /api/v1/maritim/water-area + nearest-location</t>
+          <t>GET /api/v1/maritim/route + /api/v1/maritim/water-area/water_area_point.geojson</t>
+        </is>
+      </c>
+      <c r="I27" s="20" t="inlineStr">
+        <is>
+          <t>rute pelayaran + titik area laut</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1332,12 @@
       </c>
       <c r="H28" s="20" t="inlineStr">
         <is>
-          <t>/api/v1/maps/aviation/metadata/tiles + /api/v1/sus/modelrun</t>
+          <t>GET /api/v1/maps/aviation/metadata/tiles + GET /api/v1/sus/modelrun</t>
+        </is>
+      </c>
+      <c r="I28" s="20" t="inlineStr">
+        <is>
+          <t>layer peta penerbangan + katalog run model</t>
         </is>
       </c>
     </row>
@@ -1235,7 +1366,12 @@
       </c>
       <c r="H29" s="20" t="inlineStr">
         <is>
-          <t>widis.bmkg.go.id/ndf/cgms (perlu reverse param) + inderaja HIMA (statis)</t>
+          <t>GET widis.bmkg.go.id/ndf/cgms/weather/forward</t>
+        </is>
+      </c>
+      <c r="I29" s="20" t="inlineStr">
+        <is>
+          <t>perlu reverse-engineering param; alternatif statis: inderaja HIMA</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1397,12 @@
       </c>
       <c r="H30" s="20" t="inlineStr">
         <is>
-          <t>Sama seperti r29 — belum ada endpoint JSON terdokumentasi</t>
+          <t>GET widis.bmkg.go.id/ndf/cgms/weather/forward</t>
+        </is>
+      </c>
+      <c r="I30" s="20" t="inlineStr">
+        <is>
+          <t>belum ada endpoint JSON terdokumentasi</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1428,12 @@
       </c>
       <c r="H31" s="20" t="inlineStr">
         <is>
-          <t>Sama seperti r29 — citra awan via HIMA/widis</t>
+          <t>GET widis.bmkg.go.id/ndf/cgms/weather/forward</t>
+        </is>
+      </c>
+      <c r="I31" s="20" t="inlineStr">
+        <is>
+          <t>citra awan via HIMA/widis</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1459,12 @@
       </c>
       <c r="H32" s="20" t="inlineStr">
         <is>
-          <t>Tile QPE via spartan modelrun catalog (gsmap/QPE24h)</t>
+          <t>spartan.bmkg.go.id/map/modelrun (katalog QPE/gsmap)</t>
+        </is>
+      </c>
+      <c r="I32" s="20" t="inlineStr">
+        <is>
+          <t>tile curah hujan satelit</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1490,12 @@
       </c>
       <c r="H33" s="20" t="inlineStr">
         <is>
-          <t>https://bmkg-sus.geo.id/windmap/ecmwf (wind tiles) + modelrun</t>
+          <t>GET bmkg-sus.geo.id/windmap/ecmwf</t>
+        </is>
+      </c>
+      <c r="I33" s="20" t="inlineStr">
+        <is>
+          <t>wind tiles ECMWF</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1528,12 @@
       </c>
       <c r="H34" s="20" t="inlineStr">
         <is>
-          <t>/api/v1/maps/{general,warning,maritim,aviation,tourism}/metadata/tiles</t>
+          <t>GET /api/v1/maps/{general,warning,maritim,aviation,tourism}/metadata/tiles</t>
+        </is>
+      </c>
+      <c r="I34" s="20" t="inlineStr">
+        <is>
+          <t>metadata layer peta (sources, layers, overlays)</t>
         </is>
       </c>
     </row>
@@ -1405,6 +1566,11 @@
       </c>
       <c r="H35" s="20" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I35" s="20" t="inlineStr">
+        <is>
           <t>Tidak ada di cuaca.bmkg.go.id (redesign pakai data.bmkg.go.id TEWS — legacy)</t>
         </is>
       </c>
@@ -1438,6 +1604,11 @@
       </c>
       <c r="H36" s="20" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I36" s="20" t="inlineStr">
+        <is>
           <t>Tidak ada (original redirect ke signature.bmkg.go.id/dwt)</t>
         </is>
       </c>
@@ -1462,6 +1633,11 @@
         </is>
       </c>
       <c r="H37" s="20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I37" s="20" t="inlineStr">
         <is>
           <t>Konten statis</t>
         </is>

</xml_diff>

<commit_message>
refactor(proxy): hilangkan alias /api/bmkg — path dev identik upstream; docs & xlsx pakai URL asli cuaca.bmkg.go.id
</commit_message>
<xml_diff>
--- a/docs/api-mapping/catatan-dev-team.xlsx
+++ b/docs/api-mapping/catatan-dev-team.xlsx
@@ -534,7 +534,7 @@
       </c>
       <c r="H4" s="20" t="inlineStr">
         <is>
-          <t>GET /api/df/v1/adm/coord</t>
+          <t>GET https://cuaca.bmkg.go.id/api/df/v1/adm/coord</t>
         </is>
       </c>
       <c r="I4" s="20" t="inlineStr">
@@ -572,7 +572,7 @@
       </c>
       <c r="H5" s="20" t="inlineStr">
         <is>
-          <t>GET /api/df/v1/forecast/coord</t>
+          <t>GET https://cuaca.bmkg.go.id/api/df/v1/forecast/coord</t>
         </is>
       </c>
       <c r="I5" s="20" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="H6" s="20" t="inlineStr">
         <is>
-          <t>GET /api/presentwx/coord</t>
+          <t>GET https://cuaca.bmkg.go.id/api/presentwx/coord</t>
         </is>
       </c>
       <c r="I6" s="20" t="inlineStr">
@@ -713,7 +713,7 @@
       </c>
       <c r="H9" s="20" t="inlineStr">
         <is>
-          <t>GET /api/df/v1/forecast/coord + GET /api/presentwx/coord</t>
+          <t>GET https://cuaca.bmkg.go.id/api/df/v1/forecast/coord , GET https://cuaca.bmkg.go.id/api/presentwx/coord</t>
         </is>
       </c>
       <c r="I9" s="20" t="inlineStr">
@@ -789,7 +789,7 @@
       </c>
       <c r="H11" s="20" t="inlineStr">
         <is>
-          <t>GET /api/v1/spartan/pollution/{pol}/{lvl}/{t0}/{t1}/{z}/{x}/{y}.png</t>
+          <t>GET https://cuaca.bmkg.go.id/api/v1/spartan/pollution/{pol}/{lvl}/{t0}/{t1}/{z}/{x}/{y}.png</t>
         </is>
       </c>
       <c r="I11" s="20" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="H12" s="20" t="inlineStr">
         <is>
-          <t>GET /api/presentwx/coord</t>
+          <t>GET https://cuaca.bmkg.go.id/api/presentwx/coord</t>
         </is>
       </c>
       <c r="I12" s="20" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="H13" s="20" t="inlineStr">
         <is>
-          <t>GET /api/presentwx/coord</t>
+          <t>GET https://cuaca.bmkg.go.id/api/presentwx/coord</t>
         </is>
       </c>
       <c r="I13" s="20" t="inlineStr">
@@ -885,7 +885,7 @@
       </c>
       <c r="H14" s="20" t="inlineStr">
         <is>
-          <t>GET /api/presentwx/coord</t>
+          <t>GET https://cuaca.bmkg.go.id/api/presentwx/coord</t>
         </is>
       </c>
       <c r="I14" s="20" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="H15" s="20" t="inlineStr">
         <is>
-          <t>GET /api/presentwx/coord</t>
+          <t>GET https://cuaca.bmkg.go.id/api/presentwx/coord</t>
         </is>
       </c>
       <c r="I15" s="20" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="H16" s="20" t="inlineStr">
         <is>
-          <t>GET /api/presentwx/coord</t>
+          <t>GET https://cuaca.bmkg.go.id/api/presentwx/coord</t>
         </is>
       </c>
       <c r="I16" s="20" t="inlineStr">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="H18" s="20" t="inlineStr">
         <is>
-          <t>GET /api/df/v1/forecast/coord</t>
+          <t>GET https://cuaca.bmkg.go.id/api/df/v1/forecast/coord</t>
         </is>
       </c>
       <c r="I18" s="20" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="H19" s="20" t="inlineStr">
         <is>
-          <t>GET /api/df/v1/forecast/coord</t>
+          <t>GET https://cuaca.bmkg.go.id/api/df/v1/forecast/coord</t>
         </is>
       </c>
       <c r="I19" s="20" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="H20" s="20" t="inlineStr">
         <is>
-          <t>GET /api/df/v1/forecast/coord</t>
+          <t>GET https://cuaca.bmkg.go.id/api/df/v1/forecast/coord</t>
         </is>
       </c>
       <c r="I20" s="20" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="H21" s="20" t="inlineStr">
         <is>
-          <t>GET /api/df/v1/forecast/coord</t>
+          <t>GET https://cuaca.bmkg.go.id/api/df/v1/forecast/coord</t>
         </is>
       </c>
       <c r="I21" s="20" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="H22" s="20" t="inlineStr">
         <is>
-          <t>GET /api/df/v1/forecast/coord</t>
+          <t>GET https://cuaca.bmkg.go.id/api/df/v1/forecast/coord</t>
         </is>
       </c>
       <c r="I22" s="20" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="H26" s="20" t="inlineStr">
         <is>
-          <t>GET /api/v1/public/maritim/nearest-location</t>
+          <t>GET https://cuaca.bmkg.go.id/api/v1/public/maritim/nearest-location</t>
         </is>
       </c>
       <c r="I26" s="20" t="inlineStr">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="H27" s="20" t="inlineStr">
         <is>
-          <t>GET /api/v1/maritim/route + /api/v1/maritim/water-area/water_area_point.geojson</t>
+          <t>GET https://cuaca.bmkg.go.id/api/v1/maritim/route , https://cuaca.bmkg.go.id/api/v1/maritim/water-area/water_area_point.geojson</t>
         </is>
       </c>
       <c r="I27" s="20" t="inlineStr">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="H28" s="20" t="inlineStr">
         <is>
-          <t>GET /api/v1/maps/aviation/metadata/tiles + GET /api/v1/sus/modelrun</t>
+          <t>GET https://cuaca.bmkg.go.id/api/v1/maps/aviation/metadata/tiles , GET https://cuaca.bmkg.go.id/api/v1/sus/modelrun</t>
         </is>
       </c>
       <c r="I28" s="20" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="H34" s="20" t="inlineStr">
         <is>
-          <t>GET /api/v1/maps/{general,warning,maritim,aviation,tourism}/metadata/tiles</t>
+          <t>GET https://cuaca.bmkg.go.id/api/v1/maps/{general,warning,maritim,aviation,tourism}/metadata/tiles</t>
         </is>
       </c>
       <c r="I34" s="20" t="inlineStr">

</xml_diff>

<commit_message>
docs(xlsx): prefix https:// untuk endpoint external (widis/spartan/bmkg-sus)
</commit_message>
<xml_diff>
--- a/docs/api-mapping/catatan-dev-team.xlsx
+++ b/docs/api-mapping/catatan-dev-team.xlsx
@@ -1366,7 +1366,7 @@
       </c>
       <c r="H29" s="20" t="inlineStr">
         <is>
-          <t>GET widis.bmkg.go.id/ndf/cgms/weather/forward</t>
+          <t>GET https://widis.bmkg.go.id/ndf/cgms/weather/forward</t>
         </is>
       </c>
       <c r="I29" s="20" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="H32" s="20" t="inlineStr">
         <is>
-          <t>spartan.bmkg.go.id/map/modelrun (katalog QPE/gsmap)</t>
+          <t>GET https://spartan.bmkg.go.id/map/modelrun (katalog QPE/gsmap)</t>
         </is>
       </c>
       <c r="I32" s="20" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="H33" s="20" t="inlineStr">
         <is>
-          <t>GET bmkg-sus.geo.id/windmap/ecmwf</t>
+          <t>GET https://bmkg-sus.geo.id/windmap/ecmwf</t>
         </is>
       </c>
       <c r="I33" s="20" t="inlineStr">

</xml_diff>